<commit_message>
Fix profile-total check failing after changing the number of years
The Cost/Risk Profiling "Total %" summed all 30 FY columns, so values left in
now-hidden inactive-year columns made the total != 100% and the Checks sheet
reported FAIL even when the visible active years summed to 100%.

- Total % now sums only the ACTIVE years:
  =SUM(C:INDEX(C:AF, Setup!Number-of-years)). Applied in both generators and in
  modEngine.SyncOne (so added rows match). Works in fixed and flex/dynamic modes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GMG2buRRRLJffvRsehZ8V5
</commit_message>
<xml_diff>
--- a/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
+++ b/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
@@ -3168,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="AG4" s="33">
-        <f>SUM(C4:AF4)</f>
+        <f>SUM(C4:INDEX(C4:AF4,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
         <v>0</v>
       </c>
       <c r="AG5" s="33">
-        <f>SUM(C5:AF5)</f>
+        <f>SUM(C5:INDEX(C5:AF5,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
         <v>0</v>
       </c>
       <c r="AG6" s="33">
-        <f>SUM(C6:AF6)</f>
+        <f>SUM(C6:INDEX(C6:AF6,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="AG7" s="33">
-        <f>SUM(C7:AF7)</f>
+        <f>SUM(C7:INDEX(C7:AF7,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
         <v>0</v>
       </c>
       <c r="AG8" s="33">
-        <f>SUM(C8:AF8)</f>
+        <f>SUM(C8:INDEX(C8:AF8,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
         <v>0</v>
       </c>
       <c r="AG9" s="33">
-        <f>SUM(C9:AF9)</f>
+        <f>SUM(C9:INDEX(C9:AF9,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
         <v>0</v>
       </c>
       <c r="AG4" s="33">
-        <f>SUM(C4:AF4)</f>
+        <f>SUM(C4:INDEX(C4:AF4,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="AG5" s="33">
-        <f>SUM(C5:AF5)</f>
+        <f>SUM(C5:INDEX(C5:AF5,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="AG6" s="33">
-        <f>SUM(C6:AF6)</f>
+        <f>SUM(C6:INDEX(C6:AF6,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
         <v>0</v>
       </c>
       <c r="AG7" s="33">
-        <f>SUM(C7:AF7)</f>
+        <f>SUM(C7:INDEX(C7:AF7,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix INDEX(),1,) in profile total; sequential numbering; add Delete macros
- Profile Total %: the earlier INDEX(range, N) over a horizontal range returned
  #REF! for N>1 (INDEX treated N as a row in a single-row range), so the check
  still failed. Corrected to INDEX(range, 1, N) in both generators and SyncOne.
- Cost lines now use a sequential "No." column (=ROW()-3 -> 1,2,3 …) instead of
  WBS codes; risks use ="R"&(ROW()-3) (R1,R2 …). Both auto-renumber on add/delete
  and continue correctly after existing rows.
- vba/modEngine.bas: AddCostLine/AddRisk set the auto-number formula; new
  DeleteCostLine/DeleteRisk remove the selected row (and its profiling row).
- generator: 🗑 Delete button placeholders on Cost Lines/Risk Register (D2).
- HOWTO_macros_AR.md / VBA_SETUP.md updated (delete buttons, auto-numbering).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GMG2buRRRLJffvRsehZ8V5
</commit_message>
<xml_diff>
--- a/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
+++ b/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
@@ -307,6 +307,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -326,9 +329,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1076,7 +1076,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbl_CostLines" displayName="tbl_CostLines" ref="A3:O9" headerRowCount="1">
   <autoFilter ref="A3:O9"/>
   <tableColumns count="15">
-    <tableColumn id="1" name="WBS"/>
+    <tableColumn id="1" name="No."/>
     <tableColumn id="2" name="Cost Item"/>
     <tableColumn id="3" name="Category"/>
     <tableColumn id="4" name="Description"/>
@@ -1100,7 +1100,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_CostProfile" displayName="tbl_CostProfile" ref="A3:AG9" headerRowCount="1">
   <autoFilter ref="A3:AG9"/>
   <tableColumns count="33">
-    <tableColumn id="1" name="WBS"/>
+    <tableColumn id="1" name="No."/>
     <tableColumn id="2" name="Cost Item"/>
     <tableColumn id="3" name="FY1"/>
     <tableColumn id="4" name="FY2"/>
@@ -1759,19 +1759,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Cost profile rows total 100%</t>
         </is>
@@ -1782,7 +1782,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Risk profile rows total 100%</t>
         </is>
@@ -1793,7 +1793,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Cost lines Min&lt;=ML&lt;=Max</t>
         </is>
@@ -1804,7 +1804,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Risks Min&lt;=ML&lt;=Max</t>
         </is>
@@ -1815,7 +1815,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Iterations &gt; 0</t>
         </is>
@@ -1826,7 +1826,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>Years between 1 and 30</t>
         </is>
@@ -1837,7 +1837,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Discount rate valid</t>
         </is>
@@ -2383,462 +2383,462 @@
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>➕  Add Cost Line   →  assign macro: AddCostLine</t>
+          <t>➕ Add  →  AddCostLine</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>🗑 Delete selected  →  DeleteCostLine</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>WBS</t>
-        </is>
-      </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Cost Item</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>Min Unit Cost</t>
         </is>
       </c>
-      <c r="H3" s="27" t="inlineStr">
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>Most Likely Unit Cost</t>
         </is>
       </c>
-      <c r="I3" s="27" t="inlineStr">
+      <c r="I3" s="28" t="inlineStr">
         <is>
           <t>Max Unit Cost</t>
         </is>
       </c>
-      <c r="J3" s="27" t="inlineStr">
+      <c r="J3" s="28" t="inlineStr">
         <is>
           <t>Min Total Cost</t>
         </is>
       </c>
-      <c r="K3" s="27" t="inlineStr">
+      <c r="K3" s="28" t="inlineStr">
         <is>
           <t>Most Likely Total Cost</t>
         </is>
       </c>
-      <c r="L3" s="27" t="inlineStr">
+      <c r="L3" s="28" t="inlineStr">
         <is>
           <t>Max Total Cost</t>
         </is>
       </c>
-      <c r="M3" s="27" t="inlineStr">
+      <c r="M3" s="28" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="N3" s="27" t="inlineStr">
+      <c r="N3" s="28" t="inlineStr">
         <is>
           <t>Include?</t>
         </is>
       </c>
-      <c r="O3" s="27" t="inlineStr">
+      <c r="O3" s="28" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="A4" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Site Preparation</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Civil</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Site Preparation works</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F4" s="30" t="n">
+      <c r="F4" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="G4" s="31" t="n">
         <v>28000</v>
       </c>
-      <c r="H4" s="30" t="n">
+      <c r="H4" s="31" t="n">
         <v>38000</v>
       </c>
-      <c r="I4" s="30" t="n">
+      <c r="I4" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="J4" s="31">
+      <c r="J4" s="32">
         <f>F4*G4</f>
         <v/>
       </c>
-      <c r="K4" s="31">
+      <c r="K4" s="32">
         <f>F4*H4</f>
         <v/>
       </c>
-      <c r="L4" s="31">
+      <c r="L4" s="32">
         <f>F4*I4</f>
         <v/>
       </c>
-      <c r="M4" s="28" t="inlineStr">
+      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Triangular</t>
         </is>
       </c>
-      <c r="N4" s="28" t="inlineStr">
+      <c r="N4" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O4" s="29" t="inlineStr"/>
+      <c r="O4" s="30" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="A5" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Foundations</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>Civil</t>
         </is>
       </c>
-      <c r="D5" s="29" t="inlineStr">
+      <c r="D5" s="30" t="inlineStr">
         <is>
           <t>Foundations works</t>
         </is>
       </c>
-      <c r="E5" s="28" t="inlineStr">
+      <c r="E5" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="30" t="n">
+      <c r="G5" s="31" t="n">
         <v>45000</v>
       </c>
-      <c r="H5" s="30" t="n">
+      <c r="H5" s="31" t="n">
         <v>55000</v>
       </c>
-      <c r="I5" s="30" t="n">
+      <c r="I5" s="31" t="n">
         <v>75000</v>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="32">
         <f>F5*G5</f>
         <v/>
       </c>
-      <c r="K5" s="31">
+      <c r="K5" s="32">
         <f>F5*H5</f>
         <v/>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="32">
         <f>F5*I5</f>
         <v/>
       </c>
-      <c r="M5" s="28" t="inlineStr">
+      <c r="M5" s="29" t="inlineStr">
         <is>
           <t>Triangular</t>
         </is>
       </c>
-      <c r="N5" s="28" t="inlineStr">
+      <c r="N5" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O5" s="29" t="inlineStr"/>
+      <c r="O5" s="30" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="A6" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Superstructure</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>Structural</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="30" t="inlineStr">
         <is>
           <t>Superstructure works</t>
         </is>
       </c>
-      <c r="E6" s="28" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F6" s="30" t="n">
+      <c r="F6" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="30" t="n">
+      <c r="G6" s="31" t="n">
         <v>90000</v>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="31" t="n">
         <v>120000</v>
       </c>
-      <c r="I6" s="30" t="n">
+      <c r="I6" s="31" t="n">
         <v>170000</v>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="32">
         <f>F6*G6</f>
         <v/>
       </c>
-      <c r="K6" s="31">
+      <c r="K6" s="32">
         <f>F6*H6</f>
         <v/>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="32">
         <f>F6*I6</f>
         <v/>
       </c>
-      <c r="M6" s="28" t="inlineStr">
+      <c r="M6" s="29" t="inlineStr">
         <is>
           <t>Pert</t>
         </is>
       </c>
-      <c r="N6" s="28" t="inlineStr">
+      <c r="N6" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O6" s="29" t="inlineStr"/>
+      <c r="O6" s="30" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="A7" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>MEP Systems</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>MEP</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
         <is>
           <t>MEP Systems works</t>
         </is>
       </c>
-      <c r="E7" s="28" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="31" t="n">
         <v>80000</v>
       </c>
-      <c r="I7" s="30" t="n">
+      <c r="I7" s="31" t="n">
         <v>115000</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="32">
         <f>F7*G7</f>
         <v/>
       </c>
-      <c r="K7" s="31">
+      <c r="K7" s="32">
         <f>F7*H7</f>
         <v/>
       </c>
-      <c r="L7" s="31">
+      <c r="L7" s="32">
         <f>F7*I7</f>
         <v/>
       </c>
-      <c r="M7" s="28" t="inlineStr">
+      <c r="M7" s="29" t="inlineStr">
         <is>
           <t>Pert</t>
         </is>
       </c>
-      <c r="N7" s="28" t="inlineStr">
+      <c r="N7" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O7" s="29" t="inlineStr"/>
+      <c r="O7" s="30" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="A8" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Finishes</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>Architectural</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Finishes works</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F8" s="30" t="n">
+      <c r="F8" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="30" t="n">
+      <c r="G8" s="31" t="n">
         <v>30000</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <v>45000</v>
       </c>
-      <c r="I8" s="30" t="n">
+      <c r="I8" s="31" t="n">
         <v>70000</v>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="32">
         <f>F8*G8</f>
         <v/>
       </c>
-      <c r="K8" s="31">
+      <c r="K8" s="32">
         <f>F8*H8</f>
         <v/>
       </c>
-      <c r="L8" s="31">
+      <c r="L8" s="32">
         <f>F8*I8</f>
         <v/>
       </c>
-      <c r="M8" s="28" t="inlineStr">
+      <c r="M8" s="29" t="inlineStr">
         <is>
           <t>Triangular</t>
         </is>
       </c>
-      <c r="N8" s="28" t="inlineStr">
+      <c r="N8" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O8" s="29" t="inlineStr"/>
+      <c r="O8" s="30" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="A9" s="29">
+        <f>ROW()-3</f>
+        <v/>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Project Management</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="D9" s="29" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Project Management works</t>
         </is>
       </c>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>LS</t>
         </is>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="31" t="n">
         <v>20000</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="31" t="n">
         <v>28000</v>
       </c>
-      <c r="I9" s="30" t="n">
+      <c r="I9" s="31" t="n">
         <v>40000</v>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="32">
         <f>F9*G9</f>
         <v/>
       </c>
-      <c r="K9" s="31">
+      <c r="K9" s="32">
         <f>F9*H9</f>
         <v/>
       </c>
-      <c r="L9" s="31">
+      <c r="L9" s="32">
         <f>F9*I9</f>
         <v/>
       </c>
-      <c r="M9" s="28" t="inlineStr">
+      <c r="M9" s="29" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="N9" s="28" t="inlineStr">
+      <c r="N9" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O9" s="29" t="inlineStr"/>
+      <c r="O9" s="30" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="2">
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="M4:M69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -2902,793 +2902,793 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
-        <is>
-          <t>WBS</t>
-        </is>
-      </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Cost Item</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>FY1</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>FY2</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>FY3</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>FY4</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>FY5</t>
         </is>
       </c>
-      <c r="H3" s="27" t="inlineStr">
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>FY6</t>
         </is>
       </c>
-      <c r="I3" s="27" t="inlineStr">
+      <c r="I3" s="28" t="inlineStr">
         <is>
           <t>FY7</t>
         </is>
       </c>
-      <c r="J3" s="27" t="inlineStr">
+      <c r="J3" s="28" t="inlineStr">
         <is>
           <t>FY8</t>
         </is>
       </c>
-      <c r="K3" s="27" t="inlineStr">
+      <c r="K3" s="28" t="inlineStr">
         <is>
           <t>FY9</t>
         </is>
       </c>
-      <c r="L3" s="27" t="inlineStr">
+      <c r="L3" s="28" t="inlineStr">
         <is>
           <t>FY10</t>
         </is>
       </c>
-      <c r="M3" s="27" t="inlineStr">
+      <c r="M3" s="28" t="inlineStr">
         <is>
           <t>FY11</t>
         </is>
       </c>
-      <c r="N3" s="27" t="inlineStr">
+      <c r="N3" s="28" t="inlineStr">
         <is>
           <t>FY12</t>
         </is>
       </c>
-      <c r="O3" s="27" t="inlineStr">
+      <c r="O3" s="28" t="inlineStr">
         <is>
           <t>FY13</t>
         </is>
       </c>
-      <c r="P3" s="27" t="inlineStr">
+      <c r="P3" s="28" t="inlineStr">
         <is>
           <t>FY14</t>
         </is>
       </c>
-      <c r="Q3" s="27" t="inlineStr">
+      <c r="Q3" s="28" t="inlineStr">
         <is>
           <t>FY15</t>
         </is>
       </c>
-      <c r="R3" s="27" t="inlineStr">
+      <c r="R3" s="28" t="inlineStr">
         <is>
           <t>FY16</t>
         </is>
       </c>
-      <c r="S3" s="27" t="inlineStr">
+      <c r="S3" s="28" t="inlineStr">
         <is>
           <t>FY17</t>
         </is>
       </c>
-      <c r="T3" s="27" t="inlineStr">
+      <c r="T3" s="28" t="inlineStr">
         <is>
           <t>FY18</t>
         </is>
       </c>
-      <c r="U3" s="27" t="inlineStr">
+      <c r="U3" s="28" t="inlineStr">
         <is>
           <t>FY19</t>
         </is>
       </c>
-      <c r="V3" s="27" t="inlineStr">
+      <c r="V3" s="28" t="inlineStr">
         <is>
           <t>FY20</t>
         </is>
       </c>
-      <c r="W3" s="27" t="inlineStr">
+      <c r="W3" s="28" t="inlineStr">
         <is>
           <t>FY21</t>
         </is>
       </c>
-      <c r="X3" s="27" t="inlineStr">
+      <c r="X3" s="28" t="inlineStr">
         <is>
           <t>FY22</t>
         </is>
       </c>
-      <c r="Y3" s="27" t="inlineStr">
+      <c r="Y3" s="28" t="inlineStr">
         <is>
           <t>FY23</t>
         </is>
       </c>
-      <c r="Z3" s="27" t="inlineStr">
+      <c r="Z3" s="28" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="AA3" s="27" t="inlineStr">
+      <c r="AA3" s="28" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="AB3" s="27" t="inlineStr">
+      <c r="AB3" s="28" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
       </c>
-      <c r="AC3" s="27" t="inlineStr">
+      <c r="AC3" s="28" t="inlineStr">
         <is>
           <t>FY27</t>
         </is>
       </c>
-      <c r="AD3" s="27" t="inlineStr">
+      <c r="AD3" s="28" t="inlineStr">
         <is>
           <t>FY28</t>
         </is>
       </c>
-      <c r="AE3" s="27" t="inlineStr">
+      <c r="AE3" s="28" t="inlineStr">
         <is>
           <t>FY29</t>
         </is>
       </c>
-      <c r="AF3" s="27" t="inlineStr">
+      <c r="AF3" s="28" t="inlineStr">
         <is>
           <t>FY30</t>
         </is>
       </c>
-      <c r="AG3" s="27" t="inlineStr">
+      <c r="AG3" s="28" t="inlineStr">
         <is>
           <t>Total %</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28">
+      <c r="A4" s="29">
         <f>'Cost Lines'!A4</f>
         <v/>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="30">
         <f>'Cost Lines'!B4</f>
         <v/>
       </c>
-      <c r="C4" s="32" t="n">
+      <c r="C4" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="H4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="33">
-        <f>SUM(C4:INDEX(C4:AF4,'Setup'!$C$8))</f>
+      <c r="H4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="34">
+        <f>SUM(C4:INDEX(C4:AF4,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28">
+      <c r="A5" s="29">
         <f>'Cost Lines'!A5</f>
         <v/>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="30">
         <f>'Cost Lines'!B5</f>
         <v/>
       </c>
-      <c r="C5" s="32" t="n">
+      <c r="C5" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="E5" s="32" t="n">
+      <c r="E5" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="G5" s="32" t="n">
+      <c r="G5" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="H5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="33">
-        <f>SUM(C5:INDEX(C5:AF5,'Setup'!$C$8))</f>
+      <c r="H5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="34">
+        <f>SUM(C5:INDEX(C5:AF5,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28">
+      <c r="A6" s="29">
         <f>'Cost Lines'!A6</f>
         <v/>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="30">
         <f>'Cost Lines'!B6</f>
         <v/>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="H6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="33">
-        <f>SUM(C6:INDEX(C6:AF6,'Setup'!$C$8))</f>
+      <c r="H6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="34">
+        <f>SUM(C6:INDEX(C6:AF6,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28">
+      <c r="A7" s="29">
         <f>'Cost Lines'!A7</f>
         <v/>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="30">
         <f>'Cost Lines'!B7</f>
         <v/>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="G7" s="32" t="n">
+      <c r="G7" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="H7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="33">
-        <f>SUM(C7:INDEX(C7:AF7,'Setup'!$C$8))</f>
+      <c r="H7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="34">
+        <f>SUM(C7:INDEX(C7:AF7,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28">
+      <c r="A8" s="29">
         <f>'Cost Lines'!A8</f>
         <v/>
       </c>
-      <c r="B8" s="29">
+      <c r="B8" s="30">
         <f>'Cost Lines'!B8</f>
         <v/>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="D8" s="32" t="n">
+      <c r="D8" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="H8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="33">
-        <f>SUM(C8:INDEX(C8:AF8,'Setup'!$C$8))</f>
+      <c r="H8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="34">
+        <f>SUM(C8:INDEX(C8:AF8,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28">
+      <c r="A9" s="29">
         <f>'Cost Lines'!A9</f>
         <v/>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="30">
         <f>'Cost Lines'!B9</f>
         <v/>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="32" t="n">
+      <c r="E9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="32" t="n">
+      <c r="G9" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="H9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF9" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG9" s="33">
-        <f>SUM(C9:INDEX(C9:AF9,'Setup'!$C$8))</f>
+      <c r="H9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="34">
+        <f>SUM(C9:INDEX(C9:AF9,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -3736,252 +3736,254 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="34" t="inlineStr">
-        <is>
-          <t>➕  Add Risk   →  assign macro: AddRisk</t>
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>➕ Add  →  AddRisk</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>🗑 Delete selected  →  DeleteRisk</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Risk ID</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Risk Name</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>Min Impact</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>Most Likely Impact</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>Max Impact</t>
         </is>
       </c>
-      <c r="H3" s="27" t="inlineStr">
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="I3" s="27" t="inlineStr">
+      <c r="I3" s="28" t="inlineStr">
         <is>
           <t>Risk Owner</t>
         </is>
       </c>
-      <c r="J3" s="27" t="inlineStr">
+      <c r="J3" s="28" t="inlineStr">
         <is>
           <t>Include?</t>
         </is>
       </c>
-      <c r="K3" s="27" t="inlineStr">
+      <c r="K3" s="28" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="A4" s="29">
+        <f>"R"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Adverse ground conditions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Technical</t>
         </is>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="33" t="n">
         <v>0.3</v>
       </c>
-      <c r="E4" s="30" t="n">
+      <c r="E4" s="31" t="n">
         <v>20000</v>
       </c>
-      <c r="F4" s="30" t="n">
+      <c r="F4" s="31" t="n">
         <v>45000</v>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="G4" s="31" t="n">
         <v>90000</v>
       </c>
-      <c r="H4" s="28" t="inlineStr">
+      <c r="H4" s="29" t="inlineStr">
         <is>
           <t>Triangular</t>
         </is>
       </c>
-      <c r="I4" s="29" t="inlineStr">
+      <c r="I4" s="30" t="inlineStr">
         <is>
           <t>Civil Lead</t>
         </is>
       </c>
-      <c r="J4" s="28" t="inlineStr">
+      <c r="J4" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" s="29" t="inlineStr"/>
+      <c r="K4" s="30" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
+      <c r="A5" s="29">
+        <f>"R"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>Major design change</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="31" t="n">
         <v>15000</v>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="31" t="n">
         <v>30000</v>
       </c>
-      <c r="G5" s="30" t="n">
+      <c r="G5" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="H5" s="28" t="inlineStr">
+      <c r="H5" s="29" t="inlineStr">
         <is>
           <t>Pert</t>
         </is>
       </c>
-      <c r="I5" s="29" t="inlineStr">
+      <c r="I5" s="30" t="inlineStr">
         <is>
           <t>Design Mgr</t>
         </is>
       </c>
-      <c r="J5" s="28" t="inlineStr">
+      <c r="J5" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" s="29" t="inlineStr"/>
+      <c r="K5" s="30" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="A6" s="29">
+        <f>"R"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Material price spike</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="31" t="n">
         <v>10000</v>
       </c>
-      <c r="F6" s="30" t="n">
+      <c r="F6" s="31" t="n">
         <v>25000</v>
       </c>
-      <c r="G6" s="30" t="n">
+      <c r="G6" s="31" t="n">
         <v>55000</v>
       </c>
-      <c r="H6" s="28" t="inlineStr">
+      <c r="H6" s="29" t="inlineStr">
         <is>
           <t>Triangular</t>
         </is>
       </c>
-      <c r="I6" s="29" t="inlineStr">
+      <c r="I6" s="30" t="inlineStr">
         <is>
           <t>Procurement</t>
         </is>
       </c>
-      <c r="J6" s="28" t="inlineStr">
+      <c r="J6" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" s="29" t="inlineStr"/>
+      <c r="K6" s="30" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="A7" s="29">
+        <f>"R"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Schedule delay</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="31" t="n">
         <v>20000</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>40000</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="31" t="n">
         <v>80000</v>
       </c>
-      <c r="H7" s="28" t="inlineStr">
+      <c r="H7" s="29" t="inlineStr">
         <is>
           <t>Pert</t>
         </is>
       </c>
-      <c r="I7" s="29" t="inlineStr">
+      <c r="I7" s="30" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="J7" s="28" t="inlineStr">
+      <c r="J7" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" s="29" t="inlineStr"/>
+      <c r="K7" s="30" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="2">
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="H4:H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -4045,585 +4047,585 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Risk ID</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Risk Name</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>FY1</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>FY2</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>FY3</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>FY4</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>FY5</t>
         </is>
       </c>
-      <c r="H3" s="27" t="inlineStr">
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>FY6</t>
         </is>
       </c>
-      <c r="I3" s="27" t="inlineStr">
+      <c r="I3" s="28" t="inlineStr">
         <is>
           <t>FY7</t>
         </is>
       </c>
-      <c r="J3" s="27" t="inlineStr">
+      <c r="J3" s="28" t="inlineStr">
         <is>
           <t>FY8</t>
         </is>
       </c>
-      <c r="K3" s="27" t="inlineStr">
+      <c r="K3" s="28" t="inlineStr">
         <is>
           <t>FY9</t>
         </is>
       </c>
-      <c r="L3" s="27" t="inlineStr">
+      <c r="L3" s="28" t="inlineStr">
         <is>
           <t>FY10</t>
         </is>
       </c>
-      <c r="M3" s="27" t="inlineStr">
+      <c r="M3" s="28" t="inlineStr">
         <is>
           <t>FY11</t>
         </is>
       </c>
-      <c r="N3" s="27" t="inlineStr">
+      <c r="N3" s="28" t="inlineStr">
         <is>
           <t>FY12</t>
         </is>
       </c>
-      <c r="O3" s="27" t="inlineStr">
+      <c r="O3" s="28" t="inlineStr">
         <is>
           <t>FY13</t>
         </is>
       </c>
-      <c r="P3" s="27" t="inlineStr">
+      <c r="P3" s="28" t="inlineStr">
         <is>
           <t>FY14</t>
         </is>
       </c>
-      <c r="Q3" s="27" t="inlineStr">
+      <c r="Q3" s="28" t="inlineStr">
         <is>
           <t>FY15</t>
         </is>
       </c>
-      <c r="R3" s="27" t="inlineStr">
+      <c r="R3" s="28" t="inlineStr">
         <is>
           <t>FY16</t>
         </is>
       </c>
-      <c r="S3" s="27" t="inlineStr">
+      <c r="S3" s="28" t="inlineStr">
         <is>
           <t>FY17</t>
         </is>
       </c>
-      <c r="T3" s="27" t="inlineStr">
+      <c r="T3" s="28" t="inlineStr">
         <is>
           <t>FY18</t>
         </is>
       </c>
-      <c r="U3" s="27" t="inlineStr">
+      <c r="U3" s="28" t="inlineStr">
         <is>
           <t>FY19</t>
         </is>
       </c>
-      <c r="V3" s="27" t="inlineStr">
+      <c r="V3" s="28" t="inlineStr">
         <is>
           <t>FY20</t>
         </is>
       </c>
-      <c r="W3" s="27" t="inlineStr">
+      <c r="W3" s="28" t="inlineStr">
         <is>
           <t>FY21</t>
         </is>
       </c>
-      <c r="X3" s="27" t="inlineStr">
+      <c r="X3" s="28" t="inlineStr">
         <is>
           <t>FY22</t>
         </is>
       </c>
-      <c r="Y3" s="27" t="inlineStr">
+      <c r="Y3" s="28" t="inlineStr">
         <is>
           <t>FY23</t>
         </is>
       </c>
-      <c r="Z3" s="27" t="inlineStr">
+      <c r="Z3" s="28" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
       </c>
-      <c r="AA3" s="27" t="inlineStr">
+      <c r="AA3" s="28" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
       </c>
-      <c r="AB3" s="27" t="inlineStr">
+      <c r="AB3" s="28" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
       </c>
-      <c r="AC3" s="27" t="inlineStr">
+      <c r="AC3" s="28" t="inlineStr">
         <is>
           <t>FY27</t>
         </is>
       </c>
-      <c r="AD3" s="27" t="inlineStr">
+      <c r="AD3" s="28" t="inlineStr">
         <is>
           <t>FY28</t>
         </is>
       </c>
-      <c r="AE3" s="27" t="inlineStr">
+      <c r="AE3" s="28" t="inlineStr">
         <is>
           <t>FY29</t>
         </is>
       </c>
-      <c r="AF3" s="27" t="inlineStr">
+      <c r="AF3" s="28" t="inlineStr">
         <is>
           <t>FY30</t>
         </is>
       </c>
-      <c r="AG3" s="27" t="inlineStr">
+      <c r="AG3" s="28" t="inlineStr">
         <is>
           <t>Total %</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28">
+      <c r="A4" s="29">
         <f>'Risk Register'!A4</f>
         <v/>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="30">
         <f>'Risk Register'!B4</f>
         <v/>
       </c>
-      <c r="C4" s="32" t="n">
+      <c r="C4" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="H4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="33">
-        <f>SUM(C4:INDEX(C4:AF4,'Setup'!$C$8))</f>
+      <c r="H4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="34">
+        <f>SUM(C4:INDEX(C4:AF4,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28">
+      <c r="A5" s="29">
         <f>'Risk Register'!A5</f>
         <v/>
       </c>
-      <c r="B5" s="29">
+      <c r="B5" s="30">
         <f>'Risk Register'!B5</f>
         <v/>
       </c>
-      <c r="C5" s="32" t="n">
+      <c r="C5" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="E5" s="32" t="n">
+      <c r="E5" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="G5" s="32" t="n">
+      <c r="G5" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="H5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="33">
-        <f>SUM(C5:INDEX(C5:AF5,'Setup'!$C$8))</f>
+      <c r="H5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="34">
+        <f>SUM(C5:INDEX(C5:AF5,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28">
+      <c r="A6" s="29">
         <f>'Risk Register'!A6</f>
         <v/>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="30">
         <f>'Risk Register'!B6</f>
         <v/>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>0.2222222222222222</v>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="33" t="n">
         <v>0.1111111111111111</v>
       </c>
-      <c r="H6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="33">
-        <f>SUM(C6:INDEX(C6:AF6,'Setup'!$C$8))</f>
+      <c r="H6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="34">
+        <f>SUM(C6:INDEX(C6:AF6,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28">
+      <c r="A7" s="29">
         <f>'Risk Register'!A7</f>
         <v/>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="30">
         <f>'Risk Register'!B7</f>
         <v/>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="33" t="n">
         <v>0.06666666666666667</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <v>0.1333333333333333</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.2666666666666667</v>
       </c>
-      <c r="G7" s="32" t="n">
+      <c r="G7" s="33" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="H7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="33">
-        <f>SUM(C7:INDEX(C7:AF7,'Setup'!$C$8))</f>
+      <c r="H7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="34">
+        <f>SUM(C7:INDEX(C7:AF7,1,'Setup'!$C$8))</f>
         <v/>
       </c>
     </row>
@@ -4664,29 +4666,29 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>FY</t>
         </is>
       </c>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Inflation Rate</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Cumulative Factor</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>FY1</t>
         </is>
@@ -4704,7 +4706,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>FY2</t>
         </is>
@@ -4722,7 +4724,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>FY3</t>
         </is>
@@ -4740,7 +4742,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>FY4</t>
         </is>
@@ -4758,7 +4760,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>FY5</t>
         </is>
@@ -4776,7 +4778,7 @@
       </c>
     </row>
     <row r="9" hidden="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>FY6</t>
         </is>
@@ -4794,7 +4796,7 @@
       </c>
     </row>
     <row r="10" hidden="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>FY7</t>
         </is>
@@ -4812,7 +4814,7 @@
       </c>
     </row>
     <row r="11" hidden="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>FY8</t>
         </is>
@@ -4830,7 +4832,7 @@
       </c>
     </row>
     <row r="12" hidden="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>FY9</t>
         </is>
@@ -4848,7 +4850,7 @@
       </c>
     </row>
     <row r="13" hidden="1">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>FY10</t>
         </is>
@@ -4866,7 +4868,7 @@
       </c>
     </row>
     <row r="14" hidden="1">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>FY11</t>
         </is>
@@ -4884,7 +4886,7 @@
       </c>
     </row>
     <row r="15" hidden="1">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>FY12</t>
         </is>
@@ -4902,7 +4904,7 @@
       </c>
     </row>
     <row r="16" hidden="1">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>FY13</t>
         </is>
@@ -4920,7 +4922,7 @@
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>FY14</t>
         </is>
@@ -4938,7 +4940,7 @@
       </c>
     </row>
     <row r="18" hidden="1">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>FY15</t>
         </is>
@@ -4956,7 +4958,7 @@
       </c>
     </row>
     <row r="19" hidden="1">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>FY16</t>
         </is>
@@ -4974,7 +4976,7 @@
       </c>
     </row>
     <row r="20" hidden="1">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>FY17</t>
         </is>
@@ -4992,7 +4994,7 @@
       </c>
     </row>
     <row r="21" hidden="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>FY18</t>
         </is>
@@ -5010,7 +5012,7 @@
       </c>
     </row>
     <row r="22" hidden="1">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>FY19</t>
         </is>
@@ -5028,7 +5030,7 @@
       </c>
     </row>
     <row r="23" hidden="1">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>FY20</t>
         </is>
@@ -5046,7 +5048,7 @@
       </c>
     </row>
     <row r="24" hidden="1">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>FY21</t>
         </is>
@@ -5064,7 +5066,7 @@
       </c>
     </row>
     <row r="25" hidden="1">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>FY22</t>
         </is>
@@ -5082,7 +5084,7 @@
       </c>
     </row>
     <row r="26" hidden="1">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>FY23</t>
         </is>
@@ -5100,7 +5102,7 @@
       </c>
     </row>
     <row r="27" hidden="1">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>FY24</t>
         </is>
@@ -5118,7 +5120,7 @@
       </c>
     </row>
     <row r="28" hidden="1">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>FY25</t>
         </is>
@@ -5136,7 +5138,7 @@
       </c>
     </row>
     <row r="29" hidden="1">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
@@ -5154,7 +5156,7 @@
       </c>
     </row>
     <row r="30" hidden="1">
-      <c r="A30" s="28" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>FY27</t>
         </is>
@@ -5172,7 +5174,7 @@
       </c>
     </row>
     <row r="31" hidden="1">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>FY28</t>
         </is>
@@ -5190,7 +5192,7 @@
       </c>
     </row>
     <row r="32" hidden="1">
-      <c r="A32" s="28" t="inlineStr">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>FY29</t>
         </is>
@@ -5208,7 +5210,7 @@
       </c>
     </row>
     <row r="33" hidden="1">
-      <c r="A33" s="28" t="inlineStr">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>FY30</t>
         </is>
@@ -5269,12 +5271,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Percentile</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
@@ -5286,7 +5288,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B6" s="31" t="n"/>
+      <c r="B6" s="32" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="39" t="inlineStr">
@@ -5294,7 +5296,7 @@
           <t>P30</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
+      <c r="B7" s="32" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="39" t="inlineStr">
@@ -5302,7 +5304,7 @@
           <t>P50</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n"/>
+      <c r="B8" s="32" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="39" t="inlineStr">
@@ -5310,7 +5312,7 @@
           <t>P60</t>
         </is>
       </c>
-      <c r="B9" s="31" t="n"/>
+      <c r="B9" s="32" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="39" t="inlineStr">
@@ -5318,7 +5320,7 @@
           <t>P70</t>
         </is>
       </c>
-      <c r="B10" s="31" t="n"/>
+      <c r="B10" s="32" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="39" t="inlineStr">
@@ -5326,7 +5328,7 @@
           <t>P80</t>
         </is>
       </c>
-      <c r="B11" s="31" t="n"/>
+      <c r="B11" s="32" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="39" t="inlineStr">
@@ -5334,7 +5336,7 @@
           <t>P90</t>
         </is>
       </c>
-      <c r="B12" s="31" t="n"/>
+      <c r="B12" s="32" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="39" t="inlineStr">
@@ -5342,7 +5344,7 @@
           <t>P95</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n"/>
+      <c r="B13" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -5352,27 +5354,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="28" t="inlineStr">
         <is>
           <t>Base Cost</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>Contingency</t>
         </is>
       </c>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>Contingency %</t>
         </is>
@@ -5384,9 +5386,9 @@
           <t>P50</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="31" t="n"/>
+      <c r="B17" s="32" t="n"/>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="32" t="n"/>
       <c r="E17" s="40" t="n"/>
     </row>
     <row r="18">
@@ -5395,9 +5397,9 @@
           <t>P70</t>
         </is>
       </c>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="31" t="n"/>
+      <c r="B18" s="32" t="n"/>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="32" t="n"/>
       <c r="E18" s="40" t="n"/>
     </row>
     <row r="19">
@@ -5406,9 +5408,9 @@
           <t>P80</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="31" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
       <c r="E19" s="40" t="n"/>
     </row>
     <row r="20">
@@ -5417,9 +5419,9 @@
           <t>P90</t>
         </is>
       </c>
-      <c r="B20" s="31" t="n"/>
-      <c r="C20" s="31" t="n"/>
-      <c r="D20" s="31" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
       <c r="E20" s="40" t="n"/>
     </row>
     <row r="22">
@@ -5430,27 +5432,27 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>P50</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>P70</t>
         </is>
       </c>
-      <c r="D23" s="27" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>P80</t>
         </is>
       </c>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>P90</t>
         </is>
@@ -5458,213 +5460,213 @@
     </row>
     <row r="24">
       <c r="A24" s="39" t="n"/>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="31" t="n"/>
-      <c r="D24" s="31" t="n"/>
-      <c r="E24" s="31" t="n"/>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="39" t="n"/>
-      <c r="B25" s="31" t="n"/>
-      <c r="C25" s="31" t="n"/>
-      <c r="D25" s="31" t="n"/>
-      <c r="E25" s="31" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="39" t="n"/>
-      <c r="B26" s="31" t="n"/>
-      <c r="C26" s="31" t="n"/>
-      <c r="D26" s="31" t="n"/>
-      <c r="E26" s="31" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="39" t="n"/>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="31" t="n"/>
-      <c r="D27" s="31" t="n"/>
-      <c r="E27" s="31" t="n"/>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="39" t="n"/>
-      <c r="B28" s="31" t="n"/>
-      <c r="C28" s="31" t="n"/>
-      <c r="D28" s="31" t="n"/>
-      <c r="E28" s="31" t="n"/>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="39" t="n"/>
-      <c r="B29" s="31" t="n"/>
-      <c r="C29" s="31" t="n"/>
-      <c r="D29" s="31" t="n"/>
-      <c r="E29" s="31" t="n"/>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="39" t="n"/>
-      <c r="B30" s="31" t="n"/>
-      <c r="C30" s="31" t="n"/>
-      <c r="D30" s="31" t="n"/>
-      <c r="E30" s="31" t="n"/>
+      <c r="B30" s="32" t="n"/>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="39" t="n"/>
-      <c r="B31" s="31" t="n"/>
-      <c r="C31" s="31" t="n"/>
-      <c r="D31" s="31" t="n"/>
-      <c r="E31" s="31" t="n"/>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="39" t="n"/>
-      <c r="B32" s="31" t="n"/>
-      <c r="C32" s="31" t="n"/>
-      <c r="D32" s="31" t="n"/>
-      <c r="E32" s="31" t="n"/>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="32" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="39" t="n"/>
-      <c r="B33" s="31" t="n"/>
-      <c r="C33" s="31" t="n"/>
-      <c r="D33" s="31" t="n"/>
-      <c r="E33" s="31" t="n"/>
+      <c r="B33" s="32" t="n"/>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="32" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="39" t="n"/>
-      <c r="B34" s="31" t="n"/>
-      <c r="C34" s="31" t="n"/>
-      <c r="D34" s="31" t="n"/>
-      <c r="E34" s="31" t="n"/>
+      <c r="B34" s="32" t="n"/>
+      <c r="C34" s="32" t="n"/>
+      <c r="D34" s="32" t="n"/>
+      <c r="E34" s="32" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="39" t="n"/>
-      <c r="B35" s="31" t="n"/>
-      <c r="C35" s="31" t="n"/>
-      <c r="D35" s="31" t="n"/>
-      <c r="E35" s="31" t="n"/>
+      <c r="B35" s="32" t="n"/>
+      <c r="C35" s="32" t="n"/>
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="32" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="39" t="n"/>
-      <c r="B36" s="31" t="n"/>
-      <c r="C36" s="31" t="n"/>
-      <c r="D36" s="31" t="n"/>
-      <c r="E36" s="31" t="n"/>
+      <c r="B36" s="32" t="n"/>
+      <c r="C36" s="32" t="n"/>
+      <c r="D36" s="32" t="n"/>
+      <c r="E36" s="32" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="39" t="n"/>
-      <c r="B37" s="31" t="n"/>
-      <c r="C37" s="31" t="n"/>
-      <c r="D37" s="31" t="n"/>
-      <c r="E37" s="31" t="n"/>
+      <c r="B37" s="32" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="39" t="n"/>
-      <c r="B38" s="31" t="n"/>
-      <c r="C38" s="31" t="n"/>
-      <c r="D38" s="31" t="n"/>
-      <c r="E38" s="31" t="n"/>
+      <c r="B38" s="32" t="n"/>
+      <c r="C38" s="32" t="n"/>
+      <c r="D38" s="32" t="n"/>
+      <c r="E38" s="32" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="39" t="n"/>
-      <c r="B39" s="31" t="n"/>
-      <c r="C39" s="31" t="n"/>
-      <c r="D39" s="31" t="n"/>
-      <c r="E39" s="31" t="n"/>
+      <c r="B39" s="32" t="n"/>
+      <c r="C39" s="32" t="n"/>
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="32" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="39" t="n"/>
-      <c r="B40" s="31" t="n"/>
-      <c r="C40" s="31" t="n"/>
-      <c r="D40" s="31" t="n"/>
-      <c r="E40" s="31" t="n"/>
+      <c r="B40" s="32" t="n"/>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="32" t="n"/>
+      <c r="E40" s="32" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="39" t="n"/>
-      <c r="B41" s="31" t="n"/>
-      <c r="C41" s="31" t="n"/>
-      <c r="D41" s="31" t="n"/>
-      <c r="E41" s="31" t="n"/>
+      <c r="B41" s="32" t="n"/>
+      <c r="C41" s="32" t="n"/>
+      <c r="D41" s="32" t="n"/>
+      <c r="E41" s="32" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="39" t="n"/>
-      <c r="B42" s="31" t="n"/>
-      <c r="C42" s="31" t="n"/>
-      <c r="D42" s="31" t="n"/>
-      <c r="E42" s="31" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="39" t="n"/>
-      <c r="B43" s="31" t="n"/>
-      <c r="C43" s="31" t="n"/>
-      <c r="D43" s="31" t="n"/>
-      <c r="E43" s="31" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="D43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="39" t="n"/>
-      <c r="B44" s="31" t="n"/>
-      <c r="C44" s="31" t="n"/>
-      <c r="D44" s="31" t="n"/>
-      <c r="E44" s="31" t="n"/>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="39" t="n"/>
-      <c r="B45" s="31" t="n"/>
-      <c r="C45" s="31" t="n"/>
-      <c r="D45" s="31" t="n"/>
-      <c r="E45" s="31" t="n"/>
+      <c r="B45" s="32" t="n"/>
+      <c r="C45" s="32" t="n"/>
+      <c r="D45" s="32" t="n"/>
+      <c r="E45" s="32" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="39" t="n"/>
-      <c r="B46" s="31" t="n"/>
-      <c r="C46" s="31" t="n"/>
-      <c r="D46" s="31" t="n"/>
-      <c r="E46" s="31" t="n"/>
+      <c r="B46" s="32" t="n"/>
+      <c r="C46" s="32" t="n"/>
+      <c r="D46" s="32" t="n"/>
+      <c r="E46" s="32" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="39" t="n"/>
-      <c r="B47" s="31" t="n"/>
-      <c r="C47" s="31" t="n"/>
-      <c r="D47" s="31" t="n"/>
-      <c r="E47" s="31" t="n"/>
+      <c r="B47" s="32" t="n"/>
+      <c r="C47" s="32" t="n"/>
+      <c r="D47" s="32" t="n"/>
+      <c r="E47" s="32" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="39" t="n"/>
-      <c r="B48" s="31" t="n"/>
-      <c r="C48" s="31" t="n"/>
-      <c r="D48" s="31" t="n"/>
-      <c r="E48" s="31" t="n"/>
+      <c r="B48" s="32" t="n"/>
+      <c r="C48" s="32" t="n"/>
+      <c r="D48" s="32" t="n"/>
+      <c r="E48" s="32" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="39" t="n"/>
-      <c r="B49" s="31" t="n"/>
-      <c r="C49" s="31" t="n"/>
-      <c r="D49" s="31" t="n"/>
-      <c r="E49" s="31" t="n"/>
+      <c r="B49" s="32" t="n"/>
+      <c r="C49" s="32" t="n"/>
+      <c r="D49" s="32" t="n"/>
+      <c r="E49" s="32" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="39" t="n"/>
-      <c r="B50" s="31" t="n"/>
-      <c r="C50" s="31" t="n"/>
-      <c r="D50" s="31" t="n"/>
-      <c r="E50" s="31" t="n"/>
+      <c r="B50" s="32" t="n"/>
+      <c r="C50" s="32" t="n"/>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="32" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="39" t="n"/>
-      <c r="B51" s="31" t="n"/>
-      <c r="C51" s="31" t="n"/>
-      <c r="D51" s="31" t="n"/>
-      <c r="E51" s="31" t="n"/>
+      <c r="B51" s="32" t="n"/>
+      <c r="C51" s="32" t="n"/>
+      <c r="D51" s="32" t="n"/>
+      <c r="E51" s="32" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="39" t="n"/>
-      <c r="B52" s="31" t="n"/>
-      <c r="C52" s="31" t="n"/>
-      <c r="D52" s="31" t="n"/>
-      <c r="E52" s="31" t="n"/>
+      <c r="B52" s="32" t="n"/>
+      <c r="C52" s="32" t="n"/>
+      <c r="D52" s="32" t="n"/>
+      <c r="E52" s="32" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="39" t="n"/>
-      <c r="B53" s="31" t="n"/>
-      <c r="C53" s="31" t="n"/>
-      <c r="D53" s="31" t="n"/>
-      <c r="E53" s="31" t="n"/>
+      <c r="B53" s="32" t="n"/>
+      <c r="C53" s="32" t="n"/>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="32" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -5674,17 +5676,17 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="27" t="inlineStr">
+      <c r="A57" s="28" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B57" s="27" t="inlineStr">
+      <c r="B57" s="28" t="inlineStr">
         <is>
           <t>Nominal Total</t>
         </is>
       </c>
-      <c r="C57" s="27" t="inlineStr">
+      <c r="C57" s="28" t="inlineStr">
         <is>
           <t>NPV</t>
         </is>
@@ -5696,8 +5698,8 @@
           <t>P50</t>
         </is>
       </c>
-      <c r="B58" s="31" t="n"/>
-      <c r="C58" s="31" t="n"/>
+      <c r="B58" s="32" t="n"/>
+      <c r="C58" s="32" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="39" t="inlineStr">
@@ -5705,8 +5707,8 @@
           <t>P70</t>
         </is>
       </c>
-      <c r="B59" s="31" t="n"/>
-      <c r="C59" s="31" t="n"/>
+      <c r="B59" s="32" t="n"/>
+      <c r="C59" s="32" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="39" t="inlineStr">
@@ -5714,8 +5716,8 @@
           <t>P80</t>
         </is>
       </c>
-      <c r="B60" s="31" t="n"/>
-      <c r="C60" s="31" t="n"/>
+      <c r="B60" s="32" t="n"/>
+      <c r="C60" s="32" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="39" t="inlineStr">
@@ -5723,8 +5725,8 @@
           <t>P90</t>
         </is>
       </c>
-      <c r="B61" s="31" t="n"/>
-      <c r="C61" s="31" t="n"/>
+      <c r="B61" s="32" t="n"/>
+      <c r="C61" s="32" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5763,143 +5765,143 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>P90</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>Range (P90−P10)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="n"/>
-      <c r="B5" s="29" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="31" t="n"/>
-      <c r="E5" s="31" t="n"/>
+      <c r="A5" s="30" t="n"/>
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" s="32" t="n"/>
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="32" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="n"/>
-      <c r="B6" s="29" t="n"/>
-      <c r="C6" s="31" t="n"/>
-      <c r="D6" s="31" t="n"/>
-      <c r="E6" s="31" t="n"/>
+      <c r="A6" s="30" t="n"/>
+      <c r="B6" s="30" t="n"/>
+      <c r="C6" s="32" t="n"/>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="n"/>
-      <c r="B7" s="29" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="31" t="n"/>
-      <c r="E7" s="31" t="n"/>
+      <c r="A7" s="30" t="n"/>
+      <c r="B7" s="30" t="n"/>
+      <c r="C7" s="32" t="n"/>
+      <c r="D7" s="32" t="n"/>
+      <c r="E7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="n"/>
-      <c r="B8" s="29" t="n"/>
-      <c r="C8" s="31" t="n"/>
-      <c r="D8" s="31" t="n"/>
-      <c r="E8" s="31" t="n"/>
+      <c r="A8" s="30" t="n"/>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="32" t="n"/>
+      <c r="D8" s="32" t="n"/>
+      <c r="E8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="31" t="n"/>
-      <c r="D9" s="31" t="n"/>
-      <c r="E9" s="31" t="n"/>
+      <c r="A9" s="30" t="n"/>
+      <c r="B9" s="30" t="n"/>
+      <c r="C9" s="32" t="n"/>
+      <c r="D9" s="32" t="n"/>
+      <c r="E9" s="32" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="n"/>
-      <c r="B10" s="29" t="n"/>
-      <c r="C10" s="31" t="n"/>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="31" t="n"/>
+      <c r="A10" s="30" t="n"/>
+      <c r="B10" s="30" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="n"/>
-      <c r="B11" s="29" t="n"/>
-      <c r="C11" s="31" t="n"/>
-      <c r="D11" s="31" t="n"/>
-      <c r="E11" s="31" t="n"/>
+      <c r="A11" s="30" t="n"/>
+      <c r="B11" s="30" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="n"/>
-      <c r="B12" s="29" t="n"/>
-      <c r="C12" s="31" t="n"/>
-      <c r="D12" s="31" t="n"/>
-      <c r="E12" s="31" t="n"/>
+      <c r="A12" s="30" t="n"/>
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="32" t="n"/>
+      <c r="E12" s="32" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="n"/>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="31" t="n"/>
-      <c r="D13" s="31" t="n"/>
-      <c r="E13" s="31" t="n"/>
+      <c r="A13" s="30" t="n"/>
+      <c r="B13" s="30" t="n"/>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="n"/>
-      <c r="B14" s="29" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
-      <c r="E14" s="31" t="n"/>
+      <c r="A14" s="30" t="n"/>
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="32" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="32" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n"/>
-      <c r="B15" s="29" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="31" t="n"/>
-      <c r="E15" s="31" t="n"/>
+      <c r="A15" s="30" t="n"/>
+      <c r="B15" s="30" t="n"/>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="32" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="n"/>
-      <c r="B16" s="29" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="31" t="n"/>
-      <c r="E16" s="31" t="n"/>
+      <c r="A16" s="30" t="n"/>
+      <c r="B16" s="30" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="32" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="n"/>
-      <c r="B17" s="29" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="31" t="n"/>
-      <c r="E17" s="31" t="n"/>
+      <c r="A17" s="30" t="n"/>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="32" t="n"/>
+      <c r="E17" s="32" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="n"/>
-      <c r="B18" s="29" t="n"/>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="31" t="n"/>
-      <c r="E18" s="31" t="n"/>
+      <c r="A18" s="30" t="n"/>
+      <c r="B18" s="30" t="n"/>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="32" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="n"/>
-      <c r="B19" s="29" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="31" t="n"/>
-      <c r="E19" s="31" t="n"/>
+      <c r="A19" s="30" t="n"/>
+      <c r="B19" s="30" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="n"/>
-      <c r="B20" s="29" t="n"/>
-      <c r="C20" s="31" t="n"/>
-      <c r="D20" s="31" t="n"/>
-      <c r="E20" s="31" t="n"/>
+      <c r="A20" s="30" t="n"/>
+      <c r="B20" s="30" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Make charts easy to read; default confidence P70
- Axis titles on all four Dashboard charts (cost / frequency / probability /
  year / cumulative cost / uncertainty), value-axis number formats, S-curve Y
  scaled 0-100%, and the Tornado sorted biggest-driver-first (descending in
  modEngine + reversed category axis so it's on top).
- Cumulative cash-flow chart now plots P50 and P70 (was P80).
- Default confidence level is now P70 in both workbooks (Setup + the KPIs that
  depend on it: Contingency / Recommended Budget / NPV).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GMG2buRRRLJffvRsehZ8V5
</commit_message>
<xml_diff>
--- a/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
+++ b/monte-carlo-cost-model/MonteCarloCostModel_VBA.xlsx
@@ -528,6 +528,21 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Total cost</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -541,6 +556,21 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Frequency (number of runs)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -564,7 +594,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cumulative Probability</a:t>
+              <a:t>Cumulative Probability (S-curve)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -623,12 +653,13 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Cost</a:t>
+                  <a:t>Total cost</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
@@ -637,6 +668,8 @@
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="1"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -650,12 +683,13 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Prob</a:t>
+                  <a:t>Probability (cost ≤ x)</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -763,6 +797,21 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -776,6 +825,22 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cumulative cost</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -843,7 +908,7 @@
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
+          <orientation val="maxMin"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -860,6 +925,22 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Uncertainty  (P90 − P10)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -883,7 +964,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Tornado — uncertainty drivers</a:t>
+              <a:t>Tornado — what drives the uncertainty</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -924,7 +1005,7 @@
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
+          <orientation val="maxMin"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -941,6 +1022,22 @@
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Uncertainty  (P90 − P10)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1913,7 +2010,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Cum P80</t>
+          <t>Cum P70</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2372,7 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>P80</t>
+          <t>P70</t>
         </is>
       </c>
     </row>

</xml_diff>